<commit_message>
Auditor Files: refresh document set for audit
Operator updated the Auditor Files/ tree in advance of the internal audit:
add DHRs, DHF Validations, Employee Training, Environmental Monitoring,
Equipment/Calibrations, Internal and Supplier Audits, M.SLQ001 Receiving
Inspections, Quality Objectives and Plans, and Suppliers subfolders;
replace a legacy .pptx / .dymo under DMRs/C.SLQ001 with a PDF; refresh
the CAPA, Complaints, and Management Review files.

472 files total (299 PDF, 163 DOCX, 8 XLSX, 1 DOC) at ~473 MB, all under
the 50 MB per-file preview cap.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Auditor Files/CAPA, NCMR, PCF Logs/SILQ CAPA Log.xlsx
+++ b/Auditor Files/CAPA, NCMR, PCF Logs/SILQ CAPA Log.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7ef4039dce562a81/Desktop/SilqQMS/CAPAs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7ef4039dce562a81/Desktop/SilqQMS/Auditor Files/CAPA^J NCMR^J PCF Logs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="67" documentId="13_ncr:1_{ABDB426E-FE18-EB42-9F85-E16759BC627D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78DBBD06-3E99-43F1-8F48-D2E678305D4F}"/>
+  <xr:revisionPtr revIDLastSave="69" documentId="13_ncr:1_{ABDB426E-FE18-EB42-9F85-E16759BC627D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C0CCACF-DB25-468B-8AAC-A448294864E9}"/>
   <bookViews>
-    <workbookView xWindow="28690" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="100680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2023" sheetId="9" r:id="rId1"/>
@@ -470,6 +470,8 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -497,8 +499,6 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -514,10 +514,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -807,6 +803,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE96A3F2-50F1-4A4E-8817-F5E33F62C92F}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:P35"/>
   <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="15" x14ac:dyDescent="0.4"/>
   <cols>
@@ -827,64 +826,64 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="23" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
-      <c r="K1" s="31"/>
-      <c r="L1" s="31"/>
-      <c r="M1" s="31"/>
-      <c r="N1" s="31"/>
-      <c r="O1" s="31"/>
-      <c r="P1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+      <c r="K1" s="33"/>
+      <c r="L1" s="33"/>
+      <c r="M1" s="33"/>
+      <c r="N1" s="33"/>
+      <c r="O1" s="33"/>
+      <c r="P1" s="34"/>
     </row>
     <row r="2" spans="1:16" ht="25.05" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="34"/>
-      <c r="K2" s="34"/>
-      <c r="L2" s="34"/>
-      <c r="M2" s="34"/>
-      <c r="N2" s="34"/>
-      <c r="O2" s="34"/>
-      <c r="P2" s="35"/>
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
+      <c r="H2" s="36"/>
+      <c r="I2" s="36"/>
+      <c r="J2" s="36"/>
+      <c r="K2" s="36"/>
+      <c r="L2" s="36"/>
+      <c r="M2" s="36"/>
+      <c r="N2" s="36"/>
+      <c r="O2" s="36"/>
+      <c r="P2" s="37"/>
     </row>
     <row r="3" spans="1:16" ht="15.4" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="37"/>
-      <c r="C3" s="37"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="38"/>
+      <c r="B3" s="39"/>
+      <c r="C3" s="39"/>
+      <c r="D3" s="39"/>
+      <c r="E3" s="40"/>
       <c r="F3" s="28"/>
-      <c r="G3" s="36"/>
-      <c r="H3" s="37"/>
-      <c r="I3" s="37"/>
-      <c r="J3" s="37"/>
-      <c r="K3" s="37"/>
-      <c r="L3" s="37"/>
-      <c r="M3" s="37"/>
-      <c r="N3" s="38"/>
-      <c r="O3" s="36"/>
-      <c r="P3" s="37"/>
+      <c r="G3" s="38"/>
+      <c r="H3" s="39"/>
+      <c r="I3" s="39"/>
+      <c r="J3" s="39"/>
+      <c r="K3" s="39"/>
+      <c r="L3" s="39"/>
+      <c r="M3" s="39"/>
+      <c r="N3" s="40"/>
+      <c r="O3" s="38"/>
+      <c r="P3" s="39"/>
     </row>
     <row r="4" spans="1:16" s="3" customFormat="1" ht="45" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
@@ -1012,7 +1011,7 @@
       <c r="K6" s="13">
         <v>46078</v>
       </c>
-      <c r="L6" s="39" t="s">
+      <c r="L6" s="30" t="s">
         <v>33</v>
       </c>
       <c r="M6" s="15"/>
@@ -1176,11 +1175,11 @@
       <c r="E14" s="19"/>
       <c r="F14" s="27"/>
       <c r="G14" s="20"/>
-      <c r="H14" s="40"/>
-      <c r="I14" s="40"/>
-      <c r="J14" s="40"/>
-      <c r="K14" s="40"/>
-      <c r="L14" s="40"/>
+      <c r="H14" s="31"/>
+      <c r="I14" s="31"/>
+      <c r="J14" s="31"/>
+      <c r="K14" s="31"/>
+      <c r="L14" s="31"/>
       <c r="M14" s="15"/>
       <c r="N14" s="5"/>
       <c r="O14" s="5"/>
@@ -1194,11 +1193,11 @@
       <c r="E15" s="19"/>
       <c r="F15" s="27"/>
       <c r="G15" s="20"/>
-      <c r="H15" s="40"/>
-      <c r="I15" s="40"/>
-      <c r="J15" s="40"/>
-      <c r="K15" s="40"/>
-      <c r="L15" s="40"/>
+      <c r="H15" s="31"/>
+      <c r="I15" s="31"/>
+      <c r="J15" s="31"/>
+      <c r="K15" s="31"/>
+      <c r="L15" s="31"/>
       <c r="M15" s="23"/>
       <c r="N15" s="17"/>
       <c r="O15" s="5"/>
@@ -1212,11 +1211,11 @@
       <c r="E16" s="19"/>
       <c r="F16" s="27"/>
       <c r="G16" s="20"/>
-      <c r="H16" s="40"/>
-      <c r="I16" s="40"/>
-      <c r="J16" s="40"/>
-      <c r="K16" s="40"/>
-      <c r="L16" s="40"/>
+      <c r="H16" s="31"/>
+      <c r="I16" s="31"/>
+      <c r="J16" s="31"/>
+      <c r="K16" s="31"/>
+      <c r="L16" s="31"/>
       <c r="M16" s="23"/>
       <c r="N16" s="17"/>
       <c r="O16" s="5"/>
@@ -1230,11 +1229,11 @@
       <c r="E17" s="19"/>
       <c r="F17" s="27"/>
       <c r="G17" s="20"/>
-      <c r="H17" s="40"/>
-      <c r="I17" s="40"/>
-      <c r="J17" s="40"/>
-      <c r="K17" s="40"/>
-      <c r="L17" s="40"/>
+      <c r="H17" s="31"/>
+      <c r="I17" s="31"/>
+      <c r="J17" s="31"/>
+      <c r="K17" s="31"/>
+      <c r="L17" s="31"/>
       <c r="M17" s="23"/>
       <c r="N17" s="17"/>
       <c r="O17" s="5"/>
@@ -1248,11 +1247,11 @@
       <c r="E18" s="19"/>
       <c r="F18" s="27"/>
       <c r="G18" s="20"/>
-      <c r="H18" s="40"/>
-      <c r="I18" s="40"/>
-      <c r="J18" s="40"/>
-      <c r="K18" s="40"/>
-      <c r="L18" s="40"/>
+      <c r="H18" s="31"/>
+      <c r="I18" s="31"/>
+      <c r="J18" s="31"/>
+      <c r="K18" s="31"/>
+      <c r="L18" s="31"/>
       <c r="M18" s="23"/>
       <c r="N18" s="17"/>
       <c r="O18" s="5"/>
@@ -1266,11 +1265,11 @@
       <c r="E19" s="19"/>
       <c r="F19" s="27"/>
       <c r="G19" s="20"/>
-      <c r="H19" s="40"/>
-      <c r="I19" s="40"/>
-      <c r="J19" s="40"/>
-      <c r="K19" s="40"/>
-      <c r="L19" s="40"/>
+      <c r="H19" s="31"/>
+      <c r="I19" s="31"/>
+      <c r="J19" s="31"/>
+      <c r="K19" s="31"/>
+      <c r="L19" s="31"/>
       <c r="M19" s="23"/>
       <c r="N19" s="17"/>
       <c r="O19" s="5"/>
@@ -1284,11 +1283,11 @@
       <c r="E20" s="19"/>
       <c r="F20" s="27"/>
       <c r="G20" s="20"/>
-      <c r="H20" s="40"/>
-      <c r="I20" s="40"/>
-      <c r="J20" s="40"/>
-      <c r="K20" s="40"/>
-      <c r="L20" s="40"/>
+      <c r="H20" s="31"/>
+      <c r="I20" s="31"/>
+      <c r="J20" s="31"/>
+      <c r="K20" s="31"/>
+      <c r="L20" s="31"/>
       <c r="M20" s="23"/>
       <c r="N20" s="17"/>
       <c r="O20" s="5"/>
@@ -1302,11 +1301,11 @@
       <c r="E21" s="19"/>
       <c r="F21" s="27"/>
       <c r="G21" s="20"/>
-      <c r="H21" s="40"/>
-      <c r="I21" s="40"/>
-      <c r="J21" s="40"/>
-      <c r="K21" s="40"/>
-      <c r="L21" s="40"/>
+      <c r="H21" s="31"/>
+      <c r="I21" s="31"/>
+      <c r="J21" s="31"/>
+      <c r="K21" s="31"/>
+      <c r="L21" s="31"/>
       <c r="M21" s="23"/>
       <c r="N21" s="17"/>
       <c r="O21" s="5"/>
@@ -1320,11 +1319,11 @@
       <c r="E22" s="19"/>
       <c r="F22" s="27"/>
       <c r="G22" s="20"/>
-      <c r="H22" s="40"/>
-      <c r="I22" s="40"/>
-      <c r="J22" s="40"/>
-      <c r="K22" s="40"/>
-      <c r="L22" s="40"/>
+      <c r="H22" s="31"/>
+      <c r="I22" s="31"/>
+      <c r="J22" s="31"/>
+      <c r="K22" s="31"/>
+      <c r="L22" s="31"/>
       <c r="M22" s="23"/>
       <c r="N22" s="17"/>
       <c r="O22" s="5"/>
@@ -1338,11 +1337,11 @@
       <c r="E23" s="19"/>
       <c r="F23" s="27"/>
       <c r="G23" s="20"/>
-      <c r="H23" s="40"/>
-      <c r="I23" s="40"/>
-      <c r="J23" s="40"/>
-      <c r="K23" s="40"/>
-      <c r="L23" s="40"/>
+      <c r="H23" s="31"/>
+      <c r="I23" s="31"/>
+      <c r="J23" s="31"/>
+      <c r="K23" s="31"/>
+      <c r="L23" s="31"/>
       <c r="M23" s="23"/>
       <c r="N23" s="17"/>
       <c r="O23" s="5"/>
@@ -1356,11 +1355,11 @@
       <c r="E24" s="19"/>
       <c r="F24" s="27"/>
       <c r="G24" s="20"/>
-      <c r="H24" s="40"/>
-      <c r="I24" s="40"/>
-      <c r="J24" s="40"/>
-      <c r="K24" s="40"/>
-      <c r="L24" s="40"/>
+      <c r="H24" s="31"/>
+      <c r="I24" s="31"/>
+      <c r="J24" s="31"/>
+      <c r="K24" s="31"/>
+      <c r="L24" s="31"/>
       <c r="M24" s="23"/>
       <c r="N24" s="17"/>
       <c r="O24" s="5"/>
@@ -1374,11 +1373,11 @@
       <c r="E25" s="19"/>
       <c r="F25" s="27"/>
       <c r="G25" s="20"/>
-      <c r="H25" s="40"/>
-      <c r="I25" s="40"/>
-      <c r="J25" s="40"/>
-      <c r="K25" s="40"/>
-      <c r="L25" s="40"/>
+      <c r="H25" s="31"/>
+      <c r="I25" s="31"/>
+      <c r="J25" s="31"/>
+      <c r="K25" s="31"/>
+      <c r="L25" s="31"/>
       <c r="M25" s="23"/>
       <c r="N25" s="17"/>
       <c r="O25" s="5"/>
@@ -1392,11 +1391,11 @@
       <c r="E26" s="19"/>
       <c r="F26" s="27"/>
       <c r="G26" s="20"/>
-      <c r="H26" s="40"/>
-      <c r="I26" s="40"/>
-      <c r="J26" s="40"/>
-      <c r="K26" s="40"/>
-      <c r="L26" s="40"/>
+      <c r="H26" s="31"/>
+      <c r="I26" s="31"/>
+      <c r="J26" s="31"/>
+      <c r="K26" s="31"/>
+      <c r="L26" s="31"/>
       <c r="M26" s="23"/>
       <c r="N26" s="17"/>
       <c r="O26" s="5"/>
@@ -1410,11 +1409,11 @@
       <c r="E27" s="19"/>
       <c r="F27" s="27"/>
       <c r="G27" s="20"/>
-      <c r="H27" s="40"/>
-      <c r="I27" s="40"/>
-      <c r="J27" s="40"/>
-      <c r="K27" s="40"/>
-      <c r="L27" s="40"/>
+      <c r="H27" s="31"/>
+      <c r="I27" s="31"/>
+      <c r="J27" s="31"/>
+      <c r="K27" s="31"/>
+      <c r="L27" s="31"/>
       <c r="M27" s="23"/>
       <c r="N27" s="17"/>
       <c r="O27" s="5"/>
@@ -1428,11 +1427,11 @@
       <c r="E28" s="19"/>
       <c r="F28" s="27"/>
       <c r="G28" s="20"/>
-      <c r="H28" s="40"/>
-      <c r="I28" s="40"/>
-      <c r="J28" s="40"/>
-      <c r="K28" s="40"/>
-      <c r="L28" s="40"/>
+      <c r="H28" s="31"/>
+      <c r="I28" s="31"/>
+      <c r="J28" s="31"/>
+      <c r="K28" s="31"/>
+      <c r="L28" s="31"/>
       <c r="M28" s="23"/>
       <c r="N28" s="17"/>
       <c r="O28" s="5"/>
@@ -1446,11 +1445,11 @@
       <c r="E29" s="19"/>
       <c r="F29" s="27"/>
       <c r="G29" s="20"/>
-      <c r="H29" s="40"/>
-      <c r="I29" s="40"/>
-      <c r="J29" s="40"/>
-      <c r="K29" s="40"/>
-      <c r="L29" s="40"/>
+      <c r="H29" s="31"/>
+      <c r="I29" s="31"/>
+      <c r="J29" s="31"/>
+      <c r="K29" s="31"/>
+      <c r="L29" s="31"/>
       <c r="M29" s="23"/>
       <c r="N29" s="17"/>
       <c r="O29" s="5"/>
@@ -1464,11 +1463,11 @@
       <c r="E30" s="19"/>
       <c r="F30" s="27"/>
       <c r="G30" s="20"/>
-      <c r="H30" s="40"/>
-      <c r="I30" s="40"/>
-      <c r="J30" s="40"/>
-      <c r="K30" s="40"/>
-      <c r="L30" s="40"/>
+      <c r="H30" s="31"/>
+      <c r="I30" s="31"/>
+      <c r="J30" s="31"/>
+      <c r="K30" s="31"/>
+      <c r="L30" s="31"/>
       <c r="M30" s="23"/>
       <c r="N30" s="17"/>
       <c r="O30" s="5"/>
@@ -1482,11 +1481,11 @@
       <c r="E31" s="19"/>
       <c r="F31" s="27"/>
       <c r="G31" s="20"/>
-      <c r="H31" s="40"/>
-      <c r="I31" s="40"/>
-      <c r="J31" s="40"/>
-      <c r="K31" s="40"/>
-      <c r="L31" s="40"/>
+      <c r="H31" s="31"/>
+      <c r="I31" s="31"/>
+      <c r="J31" s="31"/>
+      <c r="K31" s="31"/>
+      <c r="L31" s="31"/>
       <c r="M31" s="23"/>
       <c r="N31" s="17"/>
       <c r="O31" s="5"/>
@@ -1500,11 +1499,11 @@
       <c r="E32" s="19"/>
       <c r="F32" s="27"/>
       <c r="G32" s="20"/>
-      <c r="H32" s="40"/>
-      <c r="I32" s="40"/>
-      <c r="J32" s="40"/>
-      <c r="K32" s="40"/>
-      <c r="L32" s="40"/>
+      <c r="H32" s="31"/>
+      <c r="I32" s="31"/>
+      <c r="J32" s="31"/>
+      <c r="K32" s="31"/>
+      <c r="L32" s="31"/>
       <c r="M32" s="23"/>
       <c r="N32" s="17"/>
       <c r="O32" s="5"/>
@@ -1518,11 +1517,11 @@
       <c r="E33" s="19"/>
       <c r="F33" s="27"/>
       <c r="G33" s="20"/>
-      <c r="H33" s="40"/>
-      <c r="I33" s="40"/>
-      <c r="J33" s="40"/>
-      <c r="K33" s="40"/>
-      <c r="L33" s="40"/>
+      <c r="H33" s="31"/>
+      <c r="I33" s="31"/>
+      <c r="J33" s="31"/>
+      <c r="K33" s="31"/>
+      <c r="L33" s="31"/>
       <c r="M33" s="23"/>
       <c r="N33" s="17"/>
       <c r="O33" s="5"/>
@@ -1536,11 +1535,11 @@
       <c r="E34" s="19"/>
       <c r="F34" s="27"/>
       <c r="G34" s="20"/>
-      <c r="H34" s="40"/>
-      <c r="I34" s="40"/>
-      <c r="J34" s="40"/>
-      <c r="K34" s="40"/>
-      <c r="L34" s="40"/>
+      <c r="H34" s="31"/>
+      <c r="I34" s="31"/>
+      <c r="J34" s="31"/>
+      <c r="K34" s="31"/>
+      <c r="L34" s="31"/>
       <c r="M34" s="23"/>
       <c r="N34" s="17"/>
       <c r="O34" s="5"/>
@@ -1573,6 +1572,6 @@
     <mergeCell ref="O3:P3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="35" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <pageSetup scale="30" fitToHeight="0" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>